<commit_message>
Update roster 11/2026 from web (2 NV)
</commit_message>
<xml_diff>
--- a/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
+++ b/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN15"/>
+  <dimension ref="A1:AN13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -675,7 +675,7 @@
         <v/>
       </c>
       <c r="C12" t="str">
-        <v>Phan Như Ngọc</v>
+        <v>Phan Hiền Phúc Đạt</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -797,7 +797,7 @@
         <v/>
       </c>
       <c r="C13" t="str">
-        <v>Phan Hiền Phúc Đạt</v>
+        <v>Nguyễn Phương Linh</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -908,256 +908,12 @@
         <v>0</v>
       </c>
       <c r="AN13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v>Nguyễn Phạm Quỳnh Trang</v>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v/>
-      </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
-      <c r="H14" t="str">
-        <v/>
-      </c>
-      <c r="I14" t="str">
-        <v/>
-      </c>
-      <c r="J14" t="str">
-        <v/>
-      </c>
-      <c r="K14" t="str">
-        <v/>
-      </c>
-      <c r="L14" t="str">
-        <v/>
-      </c>
-      <c r="M14" t="str">
-        <v/>
-      </c>
-      <c r="N14" t="str">
-        <v/>
-      </c>
-      <c r="O14" t="str">
-        <v/>
-      </c>
-      <c r="P14" t="str">
-        <v/>
-      </c>
-      <c r="Q14" t="str">
-        <v/>
-      </c>
-      <c r="R14" t="str">
-        <v/>
-      </c>
-      <c r="S14" t="str">
-        <v/>
-      </c>
-      <c r="T14" t="str">
-        <v/>
-      </c>
-      <c r="U14" t="str">
-        <v/>
-      </c>
-      <c r="V14" t="str">
-        <v/>
-      </c>
-      <c r="W14" t="str">
-        <v/>
-      </c>
-      <c r="X14" t="str">
-        <v/>
-      </c>
-      <c r="Y14" t="str">
-        <v/>
-      </c>
-      <c r="Z14" t="str">
-        <v/>
-      </c>
-      <c r="AA14" t="str">
-        <v/>
-      </c>
-      <c r="AB14" t="str">
-        <v/>
-      </c>
-      <c r="AC14" t="str">
-        <v/>
-      </c>
-      <c r="AD14" t="str">
-        <v/>
-      </c>
-      <c r="AE14" t="str">
-        <v/>
-      </c>
-      <c r="AF14" t="str">
-        <v/>
-      </c>
-      <c r="AG14" t="str">
-        <v/>
-      </c>
-      <c r="AH14" t="str">
-        <v/>
-      </c>
-      <c r="AI14">
-        <v>0</v>
-      </c>
-      <c r="AJ14">
-        <v>0</v>
-      </c>
-      <c r="AK14">
-        <v>0</v>
-      </c>
-      <c r="AL14">
-        <v>0</v>
-      </c>
-      <c r="AM14">
-        <v>0</v>
-      </c>
-      <c r="AN14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v/>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <v>Nguyễn Phương Linh</v>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-      <c r="F15" t="str">
-        <v/>
-      </c>
-      <c r="G15" t="str">
-        <v/>
-      </c>
-      <c r="H15" t="str">
-        <v/>
-      </c>
-      <c r="I15" t="str">
-        <v/>
-      </c>
-      <c r="J15" t="str">
-        <v/>
-      </c>
-      <c r="K15" t="str">
-        <v/>
-      </c>
-      <c r="L15" t="str">
-        <v/>
-      </c>
-      <c r="M15" t="str">
-        <v/>
-      </c>
-      <c r="N15" t="str">
-        <v/>
-      </c>
-      <c r="O15" t="str">
-        <v/>
-      </c>
-      <c r="P15" t="str">
-        <v/>
-      </c>
-      <c r="Q15" t="str">
-        <v/>
-      </c>
-      <c r="R15" t="str">
-        <v/>
-      </c>
-      <c r="S15" t="str">
-        <v/>
-      </c>
-      <c r="T15" t="str">
-        <v/>
-      </c>
-      <c r="U15" t="str">
-        <v/>
-      </c>
-      <c r="V15" t="str">
-        <v/>
-      </c>
-      <c r="W15" t="str">
-        <v/>
-      </c>
-      <c r="X15" t="str">
-        <v/>
-      </c>
-      <c r="Y15" t="str">
-        <v/>
-      </c>
-      <c r="Z15" t="str">
-        <v/>
-      </c>
-      <c r="AA15" t="str">
-        <v/>
-      </c>
-      <c r="AB15" t="str">
-        <v/>
-      </c>
-      <c r="AC15" t="str">
-        <v/>
-      </c>
-      <c r="AD15" t="str">
-        <v/>
-      </c>
-      <c r="AE15" t="str">
-        <v/>
-      </c>
-      <c r="AF15" t="str">
-        <v/>
-      </c>
-      <c r="AG15" t="str">
-        <v/>
-      </c>
-      <c r="AH15" t="str">
-        <v/>
-      </c>
-      <c r="AI15">
-        <v>0</v>
-      </c>
-      <c r="AJ15">
-        <v>0</v>
-      </c>
-      <c r="AK15">
-        <v>0</v>
-      </c>
-      <c r="AL15">
-        <v>0</v>
-      </c>
-      <c r="AM15">
-        <v>0</v>
-      </c>
-      <c r="AN15">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 11/2026 from web (1 NV)
</commit_message>
<xml_diff>
--- a/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
+++ b/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN13"/>
+  <dimension ref="A1:AN12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -675,7 +675,7 @@
         <v/>
       </c>
       <c r="C12" t="str">
-        <v>Phan Hiền Phúc Đạt</v>
+        <v>Nguyễn Phương Linh</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -786,134 +786,12 @@
         <v>0</v>
       </c>
       <c r="AN12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v/>
-      </c>
-      <c r="B13" t="str">
-        <v/>
-      </c>
-      <c r="C13" t="str">
-        <v>Nguyễn Phương Linh</v>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13" t="str">
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
-      </c>
-      <c r="K13" t="str">
-        <v/>
-      </c>
-      <c r="L13" t="str">
-        <v/>
-      </c>
-      <c r="M13" t="str">
-        <v/>
-      </c>
-      <c r="N13" t="str">
-        <v/>
-      </c>
-      <c r="O13" t="str">
-        <v/>
-      </c>
-      <c r="P13" t="str">
-        <v/>
-      </c>
-      <c r="Q13" t="str">
-        <v/>
-      </c>
-      <c r="R13" t="str">
-        <v/>
-      </c>
-      <c r="S13" t="str">
-        <v/>
-      </c>
-      <c r="T13" t="str">
-        <v/>
-      </c>
-      <c r="U13" t="str">
-        <v/>
-      </c>
-      <c r="V13" t="str">
-        <v/>
-      </c>
-      <c r="W13" t="str">
-        <v/>
-      </c>
-      <c r="X13" t="str">
-        <v/>
-      </c>
-      <c r="Y13" t="str">
-        <v/>
-      </c>
-      <c r="Z13" t="str">
-        <v/>
-      </c>
-      <c r="AA13" t="str">
-        <v/>
-      </c>
-      <c r="AB13" t="str">
-        <v/>
-      </c>
-      <c r="AC13" t="str">
-        <v/>
-      </c>
-      <c r="AD13" t="str">
-        <v/>
-      </c>
-      <c r="AE13" t="str">
-        <v/>
-      </c>
-      <c r="AF13" t="str">
-        <v/>
-      </c>
-      <c r="AG13" t="str">
-        <v/>
-      </c>
-      <c r="AH13" t="str">
-        <v/>
-      </c>
-      <c r="AI13">
-        <v>0</v>
-      </c>
-      <c r="AJ13">
-        <v>0</v>
-      </c>
-      <c r="AK13">
-        <v>0</v>
-      </c>
-      <c r="AL13">
-        <v>0</v>
-      </c>
-      <c r="AM13">
-        <v>0</v>
-      </c>
-      <c r="AN13">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 11/2026 from web (26 NV)
</commit_message>
<xml_diff>
--- a/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
+++ b/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN33"/>
+  <dimension ref="A1:AN37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2987,13 +2987,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>DSP PQC</v>
+        <v/>
       </c>
       <c r="B31" t="str">
-        <v>41863</v>
+        <v>43311</v>
       </c>
       <c r="C31" t="str">
-        <v>Lê Ngọc Thành Tài</v>
+        <v>Đinh Minh Trí</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -3112,10 +3112,10 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>41865</v>
+        <v>43315</v>
       </c>
       <c r="C32" t="str">
-        <v>Nguyễn Đức Lộc</v>
+        <v>Huỳnh Tấn Phước</v>
       </c>
       <c r="D32" t="str">
         <v>M</v>
@@ -3234,10 +3234,10 @@
         <v/>
       </c>
       <c r="B33" t="str">
-        <v>41867</v>
+        <v>43337</v>
       </c>
       <c r="C33" t="str">
-        <v>Phan Thành Nghĩa</v>
+        <v>Vũ Trọng Khánh</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -3348,12 +3348,500 @@
         <v>0</v>
       </c>
       <c r="AN33">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v>43313</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Cù Trường Phú</v>
+      </c>
+      <c r="D34" t="str">
+        <v>E</v>
+      </c>
+      <c r="E34" t="str">
+        <v>E</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v>E</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>M</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v>M</v>
+      </c>
+      <c r="L34" t="str">
+        <v>E</v>
+      </c>
+      <c r="M34" t="str">
+        <v>E</v>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v>M</v>
+      </c>
+      <c r="P34" t="str">
+        <v>HC</v>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v>M</v>
+      </c>
+      <c r="U34" t="str">
+        <v>E</v>
+      </c>
+      <c r="V34" t="str">
+        <v>E</v>
+      </c>
+      <c r="W34" t="str">
+        <v/>
+      </c>
+      <c r="X34" t="str">
+        <v>M</v>
+      </c>
+      <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
+        <v/>
+      </c>
+      <c r="AA34" t="str">
+        <v/>
+      </c>
+      <c r="AB34" t="str">
+        <v/>
+      </c>
+      <c r="AC34" t="str">
+        <v>M</v>
+      </c>
+      <c r="AD34" t="str">
+        <v>E</v>
+      </c>
+      <c r="AE34" t="str">
+        <v/>
+      </c>
+      <c r="AF34" t="str">
+        <v>M</v>
+      </c>
+      <c r="AG34" t="str">
+        <v>NL</v>
+      </c>
+      <c r="AH34" t="str">
+        <v>M</v>
+      </c>
+      <c r="AI34">
+        <v>1</v>
+      </c>
+      <c r="AJ34">
+        <v>8</v>
+      </c>
+      <c r="AK34">
+        <v>8</v>
+      </c>
+      <c r="AL34">
+        <v>0</v>
+      </c>
+      <c r="AM34">
+        <v>1</v>
+      </c>
+      <c r="AN34">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>DSP PQC</v>
+      </c>
+      <c r="B35" t="str">
+        <v>41863</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Lê Ngọc Thành Tài</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="L35" t="str">
+        <v>E</v>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="O35" t="str">
+        <v>E</v>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="R35" t="str">
+        <v>E</v>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="U35" t="str">
+        <v>M</v>
+      </c>
+      <c r="V35" t="str">
+        <v/>
+      </c>
+      <c r="W35" t="str">
+        <v/>
+      </c>
+      <c r="X35" t="str">
+        <v/>
+      </c>
+      <c r="Y35" t="str">
+        <v/>
+      </c>
+      <c r="Z35" t="str">
+        <v>E</v>
+      </c>
+      <c r="AA35" t="str">
+        <v/>
+      </c>
+      <c r="AB35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AC35" t="str">
+        <v>E</v>
+      </c>
+      <c r="AD35" t="str">
+        <v/>
+      </c>
+      <c r="AE35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AF35" t="str">
+        <v>E</v>
+      </c>
+      <c r="AG35" t="str">
+        <v>NL</v>
+      </c>
+      <c r="AH35" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AI35">
+        <v>0</v>
+      </c>
+      <c r="AJ35">
+        <v>1</v>
+      </c>
+      <c r="AK35">
+        <v>6</v>
+      </c>
+      <c r="AL35">
+        <v>10</v>
+      </c>
+      <c r="AM35">
+        <v>1</v>
+      </c>
+      <c r="AN35">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v>41865</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Nguyễn Đức Lộc</v>
+      </c>
+      <c r="D36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="E36" t="str">
+        <v>E</v>
+      </c>
+      <c r="F36" t="str">
+        <v>E</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v>E</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="P36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="S36" t="str">
+        <v>E</v>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v>E</v>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
+      <c r="W36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="X36" t="str">
+        <v/>
+      </c>
+      <c r="Y36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="Z36" t="str">
+        <v/>
+      </c>
+      <c r="AA36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AB36" t="str">
+        <v>E</v>
+      </c>
+      <c r="AC36" t="str">
+        <v/>
+      </c>
+      <c r="AD36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AE36" t="str">
+        <v>E</v>
+      </c>
+      <c r="AF36" t="str">
+        <v/>
+      </c>
+      <c r="AG36" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AH36" t="str">
+        <v>E</v>
+      </c>
+      <c r="AI36">
+        <v>0</v>
+      </c>
+      <c r="AJ36">
+        <v>0</v>
+      </c>
+      <c r="AK36">
+        <v>8</v>
+      </c>
+      <c r="AL36">
+        <v>10</v>
+      </c>
+      <c r="AM36">
+        <v>0</v>
+      </c>
+      <c r="AN36">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v/>
+      </c>
+      <c r="B37" t="str">
+        <v>41867</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Phan Thành Nghĩa</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v>M</v>
+      </c>
+      <c r="F37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="M37" t="str">
+        <v/>
+      </c>
+      <c r="N37" t="str">
+        <v>SN</v>
+      </c>
+      <c r="O37" t="str">
+        <v/>
+      </c>
+      <c r="P37" t="str">
+        <v>E</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>E</v>
+      </c>
+      <c r="R37" t="str">
+        <v/>
+      </c>
+      <c r="S37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="T37" t="str">
+        <v>E</v>
+      </c>
+      <c r="U37" t="str">
+        <v/>
+      </c>
+      <c r="V37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="W37" t="str">
+        <v/>
+      </c>
+      <c r="X37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="Y37" t="str">
+        <v/>
+      </c>
+      <c r="Z37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AA37" t="str">
+        <v>E</v>
+      </c>
+      <c r="AB37" t="str">
+        <v/>
+      </c>
+      <c r="AC37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AD37" t="str">
+        <v>E</v>
+      </c>
+      <c r="AE37" t="str">
+        <v/>
+      </c>
+      <c r="AF37" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AG37" t="str">
+        <v>E</v>
+      </c>
+      <c r="AH37" t="str">
+        <v/>
+      </c>
+      <c r="AI37">
+        <v>0</v>
+      </c>
+      <c r="AJ37">
+        <v>1</v>
+      </c>
+      <c r="AK37">
+        <v>6</v>
+      </c>
+      <c r="AL37">
+        <v>10</v>
+      </c>
+      <c r="AM37">
+        <v>0</v>
+      </c>
+      <c r="AN37">
         <v>212</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 11/2026 from web (33 NV)
</commit_message>
<xml_diff>
--- a/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
+++ b/data/2026/11.2026/Lịch trực OCD on 11-2026 web update.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN37"/>
+  <dimension ref="A1:AN44"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3839,9 +3839,863 @@
         <v>216</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>BRF SGN</v>
+      </c>
+      <c r="B38" t="str">
+        <v>32117</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Lê Song Huyền Vi</v>
+      </c>
+      <c r="D38" t="str">
+        <v>SS</v>
+      </c>
+      <c r="E38" t="str">
+        <v>SS</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="H38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v>SS</v>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v>NC</v>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
+      <c r="R38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="S38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v>PT</v>
+      </c>
+      <c r="V38" t="str">
+        <v>PT</v>
+      </c>
+      <c r="W38" t="str">
+        <v>PT</v>
+      </c>
+      <c r="X38" t="str">
+        <v/>
+      </c>
+      <c r="Y38" t="str">
+        <v>PS</v>
+      </c>
+      <c r="Z38" t="str">
+        <v/>
+      </c>
+      <c r="AA38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AB38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AC38" t="str">
+        <v/>
+      </c>
+      <c r="AD38" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AE38" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AF38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AG38" t="str">
+        <v>HC</v>
+      </c>
+      <c r="AH38" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AI38">
+        <v>1</v>
+      </c>
+      <c r="AJ38">
+        <v>0</v>
+      </c>
+      <c r="AK38">
+        <v>0</v>
+      </c>
+      <c r="AL38">
+        <v>0</v>
+      </c>
+      <c r="AM38">
+        <v>0</v>
+      </c>
+      <c r="AN38">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v/>
+      </c>
+      <c r="B39" t="str">
+        <v>32115</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Đoàn Văn Tây</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="H39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="M39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="N39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="O39" t="str">
+        <v/>
+      </c>
+      <c r="P39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="R39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
+      <c r="T39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="U39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="V39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="W39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="X39" t="str">
+        <v/>
+      </c>
+      <c r="Y39" t="str">
+        <v/>
+      </c>
+      <c r="Z39" t="str">
+        <v/>
+      </c>
+      <c r="AA39" t="str">
+        <v/>
+      </c>
+      <c r="AB39" t="str">
+        <v/>
+      </c>
+      <c r="AC39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AD39" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AE39" t="str">
+        <v/>
+      </c>
+      <c r="AF39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AG39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AH39" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AI39">
+        <v>0</v>
+      </c>
+      <c r="AJ39">
+        <v>0</v>
+      </c>
+      <c r="AK39">
+        <v>0</v>
+      </c>
+      <c r="AL39">
+        <v>0</v>
+      </c>
+      <c r="AM39">
+        <v>0</v>
+      </c>
+      <c r="AN39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
+      <c r="B40" t="str">
+        <v>31969</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Nguyễn Thị Mỹ Hương</v>
+      </c>
+      <c r="D40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="E40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="F40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="J40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="K40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+      <c r="N40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="O40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="T40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="W40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="X40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="Y40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="Z40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AA40" t="str">
+        <v/>
+      </c>
+      <c r="AB40" t="str">
+        <v/>
+      </c>
+      <c r="AC40" t="str">
+        <v/>
+      </c>
+      <c r="AD40" t="str">
+        <v/>
+      </c>
+      <c r="AE40" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AF40" t="str">
+        <v/>
+      </c>
+      <c r="AG40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AH40" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AI40">
+        <v>0</v>
+      </c>
+      <c r="AJ40">
+        <v>0</v>
+      </c>
+      <c r="AK40">
+        <v>0</v>
+      </c>
+      <c r="AL40">
+        <v>0</v>
+      </c>
+      <c r="AM40">
+        <v>0</v>
+      </c>
+      <c r="AN40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
+      <c r="B41" t="str">
+        <v>37388</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Trương Thị Ngọc Loan</v>
+      </c>
+      <c r="D41" t="str">
+        <v>ST</v>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="J41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="K41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="L41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+      <c r="N41" t="str">
+        <v/>
+      </c>
+      <c r="O41" t="str">
+        <v>ST</v>
+      </c>
+      <c r="P41" t="str">
+        <v>ST</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>ST</v>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
+      <c r="T41" t="str">
+        <v/>
+      </c>
+      <c r="U41" t="str">
+        <v>ST</v>
+      </c>
+      <c r="V41" t="str">
+        <v/>
+      </c>
+      <c r="W41" t="str">
+        <v/>
+      </c>
+      <c r="X41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="Y41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="Z41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AA41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AB41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AC41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AD41" t="str">
+        <v/>
+      </c>
+      <c r="AE41" t="str">
+        <v>ST</v>
+      </c>
+      <c r="AF41" t="str">
+        <v/>
+      </c>
+      <c r="AG41" t="str">
+        <v>SS</v>
+      </c>
+      <c r="AH41" t="str">
+        <v/>
+      </c>
+      <c r="AI41">
+        <v>0</v>
+      </c>
+      <c r="AJ41">
+        <v>0</v>
+      </c>
+      <c r="AK41">
+        <v>0</v>
+      </c>
+      <c r="AL41">
+        <v>0</v>
+      </c>
+      <c r="AM41">
+        <v>0</v>
+      </c>
+      <c r="AN41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>BRF PQC</v>
+      </c>
+      <c r="B42" t="str">
+        <v>41366</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Phan Như Ngọc</v>
+      </c>
+      <c r="D42" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="E42" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="F42" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="G42" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v>PT</v>
+      </c>
+      <c r="K42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="L42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="M42" t="str">
+        <v/>
+      </c>
+      <c r="N42" t="str">
+        <v/>
+      </c>
+      <c r="O42" t="str">
+        <v/>
+      </c>
+      <c r="P42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="Q42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="R42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="S42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="T42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="U42" t="str">
+        <v/>
+      </c>
+      <c r="V42" t="str">
+        <v>PS</v>
+      </c>
+      <c r="W42" t="str">
+        <v/>
+      </c>
+      <c r="X42" t="str">
+        <v/>
+      </c>
+      <c r="Y42" t="str">
+        <v>PT</v>
+      </c>
+      <c r="Z42" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="AA42" t="str">
+        <v/>
+      </c>
+      <c r="AB42" t="str">
+        <v>PS</v>
+      </c>
+      <c r="AC42" t="str">
+        <v>PT</v>
+      </c>
+      <c r="AD42" t="str">
+        <v>PT</v>
+      </c>
+      <c r="AE42" t="str">
+        <v/>
+      </c>
+      <c r="AF42" t="str">
+        <v>PS</v>
+      </c>
+      <c r="AG42" t="str">
+        <v>PS</v>
+      </c>
+      <c r="AH42" t="str">
+        <v/>
+      </c>
+      <c r="AI42">
+        <v>0</v>
+      </c>
+      <c r="AJ42">
+        <v>0</v>
+      </c>
+      <c r="AK42">
+        <v>0</v>
+      </c>
+      <c r="AL42">
+        <v>0</v>
+      </c>
+      <c r="AM42">
+        <v>0</v>
+      </c>
+      <c r="AN42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v/>
+      </c>
+      <c r="B43" t="str">
+        <v>41861</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Phan Hiền Phúc Đạt</v>
+      </c>
+      <c r="D43" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="H43" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="I43" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v/>
+      </c>
+      <c r="L43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="M43" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="N43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="O43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="P43" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v>PT</v>
+      </c>
+      <c r="V43" t="str">
+        <v/>
+      </c>
+      <c r="W43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="X43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="Y43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="Z43" t="str">
+        <v/>
+      </c>
+      <c r="AA43" t="str">
+        <v>PT</v>
+      </c>
+      <c r="AB43" t="str">
+        <v>PT</v>
+      </c>
+      <c r="AC43" t="str">
+        <v/>
+      </c>
+      <c r="AD43" t="str">
+        <v/>
+      </c>
+      <c r="AE43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="AF43" t="str">
+        <v>PS</v>
+      </c>
+      <c r="AG43" t="str">
+        <v>PT</v>
+      </c>
+      <c r="AH43" t="str">
+        <v>PT</v>
+      </c>
+      <c r="AI43">
+        <v>0</v>
+      </c>
+      <c r="AJ43">
+        <v>0</v>
+      </c>
+      <c r="AK43">
+        <v>0</v>
+      </c>
+      <c r="AL43">
+        <v>0</v>
+      </c>
+      <c r="AM43">
+        <v>0</v>
+      </c>
+      <c r="AN43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v/>
+      </c>
+      <c r="B44" t="str">
+        <v>42791</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Nguyễn Phương Linh</v>
+      </c>
+      <c r="D44" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="E44" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="F44" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="I44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="J44" t="str">
+        <v>PS</v>
+      </c>
+      <c r="K44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="L44" t="str">
+        <v/>
+      </c>
+      <c r="M44" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="N44" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="O44" t="str">
+        <v>PT1</v>
+      </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="R44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="S44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="T44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="U44" t="str">
+        <v>PS</v>
+      </c>
+      <c r="V44" t="str">
+        <v/>
+      </c>
+      <c r="W44" t="str">
+        <v/>
+      </c>
+      <c r="X44" t="str">
+        <v>PT</v>
+      </c>
+      <c r="Y44" t="str">
+        <v/>
+      </c>
+      <c r="Z44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="AA44" t="str">
+        <v>PS</v>
+      </c>
+      <c r="AB44" t="str">
+        <v/>
+      </c>
+      <c r="AC44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="AD44" t="str">
+        <v/>
+      </c>
+      <c r="AE44" t="str">
+        <v/>
+      </c>
+      <c r="AF44" t="str">
+        <v/>
+      </c>
+      <c r="AG44" t="str">
+        <v>HC</v>
+      </c>
+      <c r="AH44" t="str">
+        <v>PS1</v>
+      </c>
+      <c r="AI44">
+        <v>1</v>
+      </c>
+      <c r="AJ44">
+        <v>0</v>
+      </c>
+      <c r="AK44">
+        <v>0</v>
+      </c>
+      <c r="AL44">
+        <v>0</v>
+      </c>
+      <c r="AM44">
+        <v>0</v>
+      </c>
+      <c r="AN44">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN44"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>